<commit_message>
placeholder books are now 'real' books
added and updated functions to parse book data from the csv into the bookcase view; can see call num and title on hover
</commit_message>
<xml_diff>
--- a/data/faculty_colors.xlsx
+++ b/data/faculty_colors.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tud365-my.sharepoint.com/personal/chloeedwards_tudelft_nl/Documents/Documents/GitHub/Digital-Twin-3/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="48" documentId="8_{BCE3415C-8252-468D-A9FF-9F59E6766D4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{35613AD1-391A-4573-A932-988DF2E45D57}"/>
+  <xr:revisionPtr revIDLastSave="50" documentId="8_{BCE3415C-8252-468D-A9FF-9F59E6766D4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3064727D-7CC8-47D6-94FD-AE16818653A1}"/>
   <bookViews>
-    <workbookView xWindow="18750" yWindow="-13185" windowWidth="16410" windowHeight="10035" xr2:uid="{BA0C8011-BCA6-4E61-ADCE-4985C2B159D7}"/>
+    <workbookView xWindow="-13425" yWindow="-16425" windowWidth="29040" windowHeight="15720" xr2:uid="{BA0C8011-BCA6-4E61-ADCE-4985C2B159D7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -68,9 +68,6 @@
     <t>#00B8C8</t>
   </si>
   <si>
-    <t>#E7E7E7</t>
-  </si>
-  <si>
     <t>BK</t>
   </si>
   <si>
@@ -99,6 +96,9 @@
   </si>
   <si>
     <t>#A066AA</t>
+  </si>
+  <si>
+    <t>#CFCCCC</t>
   </si>
 </sst>
 </file>
@@ -486,7 +486,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
@@ -494,15 +494,15 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B4" t="s">
         <v>4</v>
@@ -510,7 +510,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B5" t="s">
         <v>5</v>
@@ -518,7 +518,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B6" t="s">
         <v>6</v>
@@ -526,7 +526,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B7" t="s">
         <v>7</v>
@@ -534,7 +534,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B8" t="s">
         <v>8</v>
@@ -545,15 +545,15 @@
         <v>2</v>
       </c>
       <c r="B9" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>